<commit_message>
Configure GitHub Pages deployment
</commit_message>
<xml_diff>
--- a/sheet-template/plato-content-template.xlsx
+++ b/sheet-template/plato-content-template.xlsx
@@ -642,7 +642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -660,7 +660,8 @@
     <col width="28" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -741,6 +742,11 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>published</t>
         </is>
       </c>
@@ -813,7 +819,8 @@
       </c>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -891,7 +898,8 @@
           <t>Team Placeholder</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>

</xml_diff>